<commit_message>
Fill produce prices and set qty to 1 each in price list
Adds a Qty column (set to 1 for every fresh produce item) and fills
in per-kg/per-piece unit prices transcribed from the reference HOST
General Services quotation, replacing the earlier TBD placeholders.
</commit_message>
<xml_diff>
--- a/pricelist/Dhiblawe-Trading-Product-Price-List.xlsx
+++ b/pricelist/Dhiblawe-Trading-Product-Price-List.xlsx
@@ -105,7 +105,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="6">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -149,17 +149,6 @@
     </border>
     <border>
       <left/>
-      <right/>
-      <top style="thin">
-        <color rgb="00E3E6EB"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="00E3E6EB"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
       <right style="thin">
         <color rgb="00E3E6EB"/>
       </right>
@@ -175,7 +164,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -219,7 +208,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -586,7 +574,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F50"/>
+  <dimension ref="A1:F51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -633,7 +621,7 @@
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>All prices in US Dollars (USD). Prices marked “TBD” are placeholders pending confirmation.</t>
+          <t>All prices in US Dollars (USD), per unit (kg or piece as noted).</t>
         </is>
       </c>
     </row>
@@ -979,13 +967,17 @@
           <t>Unit</t>
         </is>
       </c>
-      <c r="D21" s="15" t="inlineStr">
+      <c r="D21" s="10" t="inlineStr">
+        <is>
+          <t>Qty</t>
+        </is>
+      </c>
+      <c r="E21" s="15" t="inlineStr">
         <is>
           <t>Unit Price</t>
         </is>
       </c>
-      <c r="E21" s="16" t="n"/>
-      <c r="F21" s="17" t="n"/>
+      <c r="F21" s="16" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="11" t="n">
@@ -1001,12 +993,14 @@
           <t>Pc</t>
         </is>
       </c>
-      <c r="D22" s="11" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="E22" s="11" t="n"/>
+      <c r="D22" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="E22" s="11" t="inlineStr">
+        <is>
+          <t>$ 2.60</t>
+        </is>
+      </c>
       <c r="F22" s="11" t="n"/>
     </row>
     <row r="23">
@@ -1023,12 +1017,14 @@
           <t>Kg</t>
         </is>
       </c>
-      <c r="D23" s="13" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="E23" s="13" t="n"/>
+      <c r="D23" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="E23" s="13" t="inlineStr">
+        <is>
+          <t>$ 4.00</t>
+        </is>
+      </c>
       <c r="F23" s="13" t="n"/>
     </row>
     <row r="24">
@@ -1045,12 +1041,14 @@
           <t>Kg</t>
         </is>
       </c>
-      <c r="D24" s="11" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="E24" s="11" t="n"/>
+      <c r="D24" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="E24" s="11" t="inlineStr">
+        <is>
+          <t>$ 3.00</t>
+        </is>
+      </c>
       <c r="F24" s="11" t="n"/>
     </row>
     <row r="25">
@@ -1067,12 +1065,14 @@
           <t>Kg</t>
         </is>
       </c>
-      <c r="D25" s="13" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="E25" s="13" t="n"/>
+      <c r="D25" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="E25" s="13" t="inlineStr">
+        <is>
+          <t>$ 3.00</t>
+        </is>
+      </c>
       <c r="F25" s="13" t="n"/>
     </row>
     <row r="26">
@@ -1089,12 +1089,14 @@
           <t>Kg</t>
         </is>
       </c>
-      <c r="D26" s="11" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="E26" s="11" t="n"/>
+      <c r="D26" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="E26" s="11" t="inlineStr">
+        <is>
+          <t>$ 8.00</t>
+        </is>
+      </c>
       <c r="F26" s="11" t="n"/>
     </row>
     <row r="27">
@@ -1111,12 +1113,14 @@
           <t>Kg</t>
         </is>
       </c>
-      <c r="D27" s="13" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="E27" s="13" t="n"/>
+      <c r="D27" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="E27" s="13" t="inlineStr">
+        <is>
+          <t>$ 2.00</t>
+        </is>
+      </c>
       <c r="F27" s="13" t="n"/>
     </row>
     <row r="28">
@@ -1133,12 +1137,14 @@
           <t>Kg</t>
         </is>
       </c>
-      <c r="D28" s="11" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="E28" s="11" t="n"/>
+      <c r="D28" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="E28" s="11" t="inlineStr">
+        <is>
+          <t>$ 3.00</t>
+        </is>
+      </c>
       <c r="F28" s="11" t="n"/>
     </row>
     <row r="29">
@@ -1155,12 +1161,14 @@
           <t>Kg</t>
         </is>
       </c>
-      <c r="D29" s="13" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="E29" s="13" t="n"/>
+      <c r="D29" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="E29" s="13" t="inlineStr">
+        <is>
+          <t>$ 3.00</t>
+        </is>
+      </c>
       <c r="F29" s="13" t="n"/>
     </row>
     <row r="30">
@@ -1177,12 +1185,14 @@
           <t>Kg</t>
         </is>
       </c>
-      <c r="D30" s="11" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="E30" s="11" t="n"/>
+      <c r="D30" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="E30" s="11" t="inlineStr">
+        <is>
+          <t>$ 3.00</t>
+        </is>
+      </c>
       <c r="F30" s="11" t="n"/>
     </row>
     <row r="31">
@@ -1199,12 +1209,14 @@
           <t>Kg</t>
         </is>
       </c>
-      <c r="D31" s="13" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="E31" s="13" t="n"/>
+      <c r="D31" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="E31" s="13" t="inlineStr">
+        <is>
+          <t>$ 7.00</t>
+        </is>
+      </c>
       <c r="F31" s="13" t="n"/>
     </row>
     <row r="32">
@@ -1221,12 +1233,14 @@
           <t>Kg</t>
         </is>
       </c>
-      <c r="D32" s="11" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="E32" s="11" t="n"/>
+      <c r="D32" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="E32" s="11" t="inlineStr">
+        <is>
+          <t>$ 4.50</t>
+        </is>
+      </c>
       <c r="F32" s="11" t="n"/>
     </row>
     <row r="33">
@@ -1243,12 +1257,14 @@
           <t>Kg</t>
         </is>
       </c>
-      <c r="D33" s="13" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="E33" s="13" t="n"/>
+      <c r="D33" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="E33" s="13" t="inlineStr">
+        <is>
+          <t>$ 5.50</t>
+        </is>
+      </c>
       <c r="F33" s="13" t="n"/>
     </row>
     <row r="34">
@@ -1265,12 +1281,14 @@
           <t>Kg</t>
         </is>
       </c>
-      <c r="D34" s="11" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="E34" s="11" t="n"/>
+      <c r="D34" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="E34" s="11" t="inlineStr">
+        <is>
+          <t>$ 5.00</t>
+        </is>
+      </c>
       <c r="F34" s="11" t="n"/>
     </row>
     <row r="35">
@@ -1287,12 +1305,14 @@
           <t>Kg</t>
         </is>
       </c>
-      <c r="D35" s="13" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="E35" s="13" t="n"/>
+      <c r="D35" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="E35" s="13" t="inlineStr">
+        <is>
+          <t>$ 4.00</t>
+        </is>
+      </c>
       <c r="F35" s="13" t="n"/>
     </row>
     <row r="36">
@@ -1309,12 +1329,14 @@
           <t>Kg</t>
         </is>
       </c>
-      <c r="D36" s="11" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="E36" s="11" t="n"/>
+      <c r="D36" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="E36" s="11" t="inlineStr">
+        <is>
+          <t>$ 4.00</t>
+        </is>
+      </c>
       <c r="F36" s="11" t="n"/>
     </row>
     <row r="37">
@@ -1331,12 +1353,14 @@
           <t>Kg</t>
         </is>
       </c>
-      <c r="D37" s="13" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="E37" s="13" t="n"/>
+      <c r="D37" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="E37" s="13" t="inlineStr">
+        <is>
+          <t>$ 3.00</t>
+        </is>
+      </c>
       <c r="F37" s="13" t="n"/>
     </row>
     <row r="38">
@@ -1353,12 +1377,14 @@
           <t>Kg</t>
         </is>
       </c>
-      <c r="D38" s="11" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="E38" s="11" t="n"/>
+      <c r="D38" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="E38" s="11" t="inlineStr">
+        <is>
+          <t>$ 5.00</t>
+        </is>
+      </c>
       <c r="F38" s="11" t="n"/>
     </row>
     <row r="39">
@@ -1375,12 +1401,14 @@
           <t>Kg</t>
         </is>
       </c>
-      <c r="D39" s="13" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="E39" s="13" t="n"/>
+      <c r="D39" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="E39" s="13" t="inlineStr">
+        <is>
+          <t>$ 4.00</t>
+        </is>
+      </c>
       <c r="F39" s="13" t="n"/>
     </row>
     <row r="40">
@@ -1397,12 +1425,14 @@
           <t>Kg</t>
         </is>
       </c>
-      <c r="D40" s="11" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="E40" s="11" t="n"/>
+      <c r="D40" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="E40" s="11" t="inlineStr">
+        <is>
+          <t>$ 2.50</t>
+        </is>
+      </c>
       <c r="F40" s="11" t="n"/>
     </row>
     <row r="41">
@@ -1419,12 +1449,14 @@
           <t>Kg</t>
         </is>
       </c>
-      <c r="D41" s="13" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="E41" s="13" t="n"/>
+      <c r="D41" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="E41" s="13" t="inlineStr">
+        <is>
+          <t>$ 3.30</t>
+        </is>
+      </c>
       <c r="F41" s="13" t="n"/>
     </row>
     <row r="42">
@@ -1441,12 +1473,14 @@
           <t>Kg</t>
         </is>
       </c>
-      <c r="D42" s="11" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="E42" s="11" t="n"/>
+      <c r="D42" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="E42" s="11" t="inlineStr">
+        <is>
+          <t>$ 6.00</t>
+        </is>
+      </c>
       <c r="F42" s="11" t="n"/>
     </row>
     <row r="43">
@@ -1463,12 +1497,14 @@
           <t>Kg</t>
         </is>
       </c>
-      <c r="D43" s="13" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="E43" s="13" t="n"/>
+      <c r="D43" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="E43" s="13" t="inlineStr">
+        <is>
+          <t>$ 4.00</t>
+        </is>
+      </c>
       <c r="F43" s="13" t="n"/>
     </row>
     <row r="44">
@@ -1485,12 +1521,14 @@
           <t>Kg</t>
         </is>
       </c>
-      <c r="D44" s="11" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="E44" s="11" t="n"/>
+      <c r="D44" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="E44" s="11" t="inlineStr">
+        <is>
+          <t>$ 3.00</t>
+        </is>
+      </c>
       <c r="F44" s="11" t="n"/>
     </row>
     <row r="47">
@@ -1501,7 +1539,7 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="18" t="inlineStr">
+      <c r="A48" s="17" t="inlineStr">
         <is>
           <t>•</t>
         </is>
@@ -1513,66 +1551,79 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="18" t="inlineStr">
+      <c r="A49" s="17" t="inlineStr">
         <is>
           <t>•</t>
         </is>
       </c>
       <c r="B49" s="3" t="inlineStr">
         <is>
-          <t>Fresh produce items are sourced from Dhiblawe Trading’s regular supply line; unit prices marked “TBD” to be confirmed before quoting to a customer.</t>
+          <t>Fresh produce unit prices (per kg or per piece) are shown for a reference quantity of 1; multiply by the order quantity for a line total.</t>
         </is>
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="18" t="inlineStr">
+      <c r="A50" s="17" t="inlineStr">
         <is>
           <t>•</t>
         </is>
       </c>
       <c r="B50" s="3" t="inlineStr">
         <is>
+          <t>Produce prices were transcribed from a reference quotation image — please double-check figures before quoting a customer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="17" t="inlineStr">
+        <is>
+          <t>•</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="inlineStr">
+        <is>
           <t>Prices exclude delivery, customs, and handling unless otherwise agreed.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="35">
-    <mergeCell ref="D27:F27"/>
-    <mergeCell ref="D41:F41"/>
-    <mergeCell ref="D32:F32"/>
+  <mergeCells count="36">
+    <mergeCell ref="E43:F43"/>
+    <mergeCell ref="E24:F24"/>
+    <mergeCell ref="E33:F33"/>
+    <mergeCell ref="E42:F42"/>
+    <mergeCell ref="E23:F23"/>
     <mergeCell ref="A3:F3"/>
-    <mergeCell ref="D43:F43"/>
+    <mergeCell ref="E39:F39"/>
+    <mergeCell ref="E44:F44"/>
     <mergeCell ref="A2:F2"/>
-    <mergeCell ref="D28:F28"/>
+    <mergeCell ref="E35:F35"/>
     <mergeCell ref="A47:F47"/>
-    <mergeCell ref="D37:F37"/>
+    <mergeCell ref="E38:F38"/>
+    <mergeCell ref="E29:F29"/>
     <mergeCell ref="B48:F48"/>
     <mergeCell ref="A5:F5"/>
     <mergeCell ref="A8:F8"/>
-    <mergeCell ref="D30:F30"/>
-    <mergeCell ref="D25:F25"/>
+    <mergeCell ref="E28:F28"/>
     <mergeCell ref="A20:F20"/>
-    <mergeCell ref="D39:F39"/>
-    <mergeCell ref="D33:F33"/>
-    <mergeCell ref="D24:F24"/>
-    <mergeCell ref="D42:F42"/>
-    <mergeCell ref="D38:F38"/>
-    <mergeCell ref="D29:F29"/>
-    <mergeCell ref="D23:F23"/>
-    <mergeCell ref="D35:F35"/>
-    <mergeCell ref="D26:F26"/>
-    <mergeCell ref="D44:F44"/>
-    <mergeCell ref="D34:F34"/>
+    <mergeCell ref="E40:F40"/>
+    <mergeCell ref="E31:F31"/>
+    <mergeCell ref="E34:F34"/>
+    <mergeCell ref="E30:F30"/>
+    <mergeCell ref="E27:F27"/>
+    <mergeCell ref="E36:F36"/>
+    <mergeCell ref="E26:F26"/>
     <mergeCell ref="B49:F49"/>
-    <mergeCell ref="D31:F31"/>
+    <mergeCell ref="E32:F32"/>
+    <mergeCell ref="E25:F25"/>
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="D22:F22"/>
-    <mergeCell ref="D40:F40"/>
-    <mergeCell ref="D36:F36"/>
+    <mergeCell ref="E41:F41"/>
+    <mergeCell ref="B51:F51"/>
     <mergeCell ref="A6:F6"/>
-    <mergeCell ref="D21:F21"/>
+    <mergeCell ref="E37:F37"/>
+    <mergeCell ref="E22:F22"/>
     <mergeCell ref="B50:F50"/>
+    <mergeCell ref="E21:F21"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>